<commit_message>
MEGA update - Final version
</commit_message>
<xml_diff>
--- a/2. Documentation/0. Project Details/Timeline.xlsx
+++ b/2. Documentation/0. Project Details/Timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fc6206cd76c8efb5/Documents/SCHOOL_TECH/1-Current Courses/Capstone I/1. Git Repo/S26_Team6_LaniEV-RetroFit/2. Documentation/0. Project Details/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{09987254-AD0E-4C28-A73A-9075852F49BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1402EFFE-03D3-46A1-9365-CC7FB34A3BAE}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{09987254-AD0E-4C28-A73A-9075852F49BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{889F6AD3-F823-4C9E-B313-32021DB2F0C4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Insert new rows ABOVE this one</t>
   </si>
@@ -125,12 +125,6 @@
     <t>Alec Snodgrass</t>
   </si>
   <si>
-    <t>Team Contract</t>
-  </si>
-  <si>
-    <t>Project Proposal</t>
-  </si>
-  <si>
     <t>Conceptual Design</t>
   </si>
   <si>
@@ -141,6 +135,15 @@
   </si>
   <si>
     <t>DURATION (days)</t>
+  </si>
+  <si>
+    <t>Initial Vehicle Report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery Conversion Manual </t>
+  </si>
+  <si>
+    <t>Wiring Schematic</t>
   </si>
 </sst>
 </file>
@@ -720,7 +723,7 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -938,13 +941,19 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="166" fontId="14" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="14" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="14" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -968,7 +977,61 @@
     <cellStyle name="Title" xfId="4" builtinId="15" customBuiltin="1"/>
     <cellStyle name="zHiddenText" xfId="2" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="26">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1002,15 +1065,35 @@
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
       <border>
-        <left style="thin">
-          <color theme="5"/>
-        </left>
-        <right style="thin">
-          <color theme="5"/>
-        </right>
-        <vertical/>
-        <horizontal/>
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0" tint="-4.9989318521683403E-2"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1126,6 +1209,18 @@
     <dxf>
       <border>
         <left style="thin">
+          <color theme="5"/>
+        </left>
+        <right style="thin">
+          <color theme="5"/>
+        </right>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
           <color theme="0" tint="-0.24994659260841701"/>
         </left>
       </border>
@@ -1219,15 +1314,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ToDoList" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="19"/>
-      <tableStyleElement type="headerRow" dxfId="18"/>
-      <tableStyleElement type="totalRow" dxfId="17"/>
-      <tableStyleElement type="firstColumn" dxfId="16"/>
-      <tableStyleElement type="lastColumn" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="secondRowStripe" dxfId="13"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="12"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="11"/>
+      <tableStyleElement type="wholeTable" dxfId="25"/>
+      <tableStyleElement type="headerRow" dxfId="24"/>
+      <tableStyleElement type="totalRow" dxfId="23"/>
+      <tableStyleElement type="firstColumn" dxfId="22"/>
+      <tableStyleElement type="lastColumn" dxfId="21"/>
+      <tableStyleElement type="firstRowStripe" dxfId="20"/>
+      <tableStyleElement type="secondRowStripe" dxfId="19"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="18"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="17"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1582,7 +1677,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DO16"/>
+  <dimension ref="A1:DO18"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.69921875" style="12" customWidth="1"/>
@@ -1615,7 +1710,7 @@
       <c r="N1" s="79"/>
       <c r="O1" s="18"/>
       <c r="P1" s="77">
-        <v>46050</v>
+        <v>46108</v>
       </c>
       <c r="Q1" s="76"/>
       <c r="R1" s="76"/>
@@ -1672,166 +1767,166 @@
       <c r="D4" s="67"/>
       <c r="E4" s="68"/>
       <c r="F4" s="68"/>
-      <c r="H4" s="83">
+      <c r="H4" s="82">
         <f>H5</f>
-        <v>46048</v>
-      </c>
-      <c r="I4" s="81"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
+        <v>46104</v>
+      </c>
+      <c r="I4" s="82"/>
+      <c r="J4" s="82"/>
+      <c r="K4" s="82"/>
+      <c r="L4" s="82"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="84"/>
       <c r="O4" s="81">
         <f>O5</f>
-        <v>46055</v>
-      </c>
-      <c r="P4" s="81"/>
-      <c r="Q4" s="81"/>
-      <c r="R4" s="81"/>
-      <c r="S4" s="81"/>
-      <c r="T4" s="81"/>
-      <c r="U4" s="81"/>
+        <v>46111</v>
+      </c>
+      <c r="P4" s="82"/>
+      <c r="Q4" s="82"/>
+      <c r="R4" s="82"/>
+      <c r="S4" s="82"/>
+      <c r="T4" s="82"/>
+      <c r="U4" s="84"/>
       <c r="V4" s="81">
         <f>V5</f>
-        <v>46062</v>
-      </c>
-      <c r="W4" s="81"/>
-      <c r="X4" s="81"/>
-      <c r="Y4" s="81"/>
-      <c r="Z4" s="81"/>
-      <c r="AA4" s="81"/>
-      <c r="AB4" s="81"/>
+        <v>46118</v>
+      </c>
+      <c r="W4" s="82"/>
+      <c r="X4" s="82"/>
+      <c r="Y4" s="82"/>
+      <c r="Z4" s="82"/>
+      <c r="AA4" s="82"/>
+      <c r="AB4" s="84"/>
       <c r="AC4" s="81">
         <f>AC5</f>
-        <v>46069</v>
-      </c>
-      <c r="AD4" s="81"/>
-      <c r="AE4" s="81"/>
-      <c r="AF4" s="81"/>
-      <c r="AG4" s="81"/>
-      <c r="AH4" s="81"/>
-      <c r="AI4" s="81"/>
+        <v>46125</v>
+      </c>
+      <c r="AD4" s="82"/>
+      <c r="AE4" s="82"/>
+      <c r="AF4" s="82"/>
+      <c r="AG4" s="82"/>
+      <c r="AH4" s="82"/>
+      <c r="AI4" s="84"/>
       <c r="AJ4" s="81">
         <f>AJ5</f>
-        <v>46076</v>
-      </c>
-      <c r="AK4" s="81"/>
-      <c r="AL4" s="81"/>
-      <c r="AM4" s="81"/>
-      <c r="AN4" s="81"/>
-      <c r="AO4" s="81"/>
-      <c r="AP4" s="81"/>
+        <v>46132</v>
+      </c>
+      <c r="AK4" s="82"/>
+      <c r="AL4" s="82"/>
+      <c r="AM4" s="82"/>
+      <c r="AN4" s="82"/>
+      <c r="AO4" s="82"/>
+      <c r="AP4" s="84"/>
       <c r="AQ4" s="81">
         <f>AQ5</f>
-        <v>46083</v>
-      </c>
-      <c r="AR4" s="81"/>
-      <c r="AS4" s="81"/>
-      <c r="AT4" s="81"/>
-      <c r="AU4" s="81"/>
-      <c r="AV4" s="81"/>
-      <c r="AW4" s="81"/>
+        <v>46139</v>
+      </c>
+      <c r="AR4" s="82"/>
+      <c r="AS4" s="82"/>
+      <c r="AT4" s="82"/>
+      <c r="AU4" s="82"/>
+      <c r="AV4" s="82"/>
+      <c r="AW4" s="84"/>
       <c r="AX4" s="81">
         <f>AX5</f>
-        <v>46090</v>
-      </c>
-      <c r="AY4" s="81"/>
-      <c r="AZ4" s="81"/>
-      <c r="BA4" s="81"/>
-      <c r="BB4" s="81"/>
-      <c r="BC4" s="81"/>
-      <c r="BD4" s="81"/>
+        <v>46146</v>
+      </c>
+      <c r="AY4" s="82"/>
+      <c r="AZ4" s="82"/>
+      <c r="BA4" s="82"/>
+      <c r="BB4" s="82"/>
+      <c r="BC4" s="82"/>
+      <c r="BD4" s="84"/>
       <c r="BE4" s="81">
         <f>BE5</f>
-        <v>46097</v>
-      </c>
-      <c r="BF4" s="81"/>
-      <c r="BG4" s="81"/>
-      <c r="BH4" s="81"/>
-      <c r="BI4" s="81"/>
-      <c r="BJ4" s="81"/>
-      <c r="BK4" s="82"/>
-      <c r="BL4" s="85">
+        <v>46153</v>
+      </c>
+      <c r="BF4" s="82"/>
+      <c r="BG4" s="82"/>
+      <c r="BH4" s="82"/>
+      <c r="BI4" s="82"/>
+      <c r="BJ4" s="82"/>
+      <c r="BK4" s="83"/>
+      <c r="BL4" s="87">
         <f>BL5</f>
-        <v>46104</v>
-      </c>
-      <c r="BM4" s="81"/>
-      <c r="BN4" s="81"/>
-      <c r="BO4" s="81"/>
-      <c r="BP4" s="81"/>
-      <c r="BQ4" s="81"/>
-      <c r="BR4" s="81"/>
-      <c r="BS4" s="81">
+        <v>46160</v>
+      </c>
+      <c r="BM4" s="85"/>
+      <c r="BN4" s="85"/>
+      <c r="BO4" s="85"/>
+      <c r="BP4" s="85"/>
+      <c r="BQ4" s="85"/>
+      <c r="BR4" s="85"/>
+      <c r="BS4" s="85">
         <f>BS5</f>
-        <v>46111</v>
-      </c>
-      <c r="BT4" s="81"/>
-      <c r="BU4" s="81"/>
-      <c r="BV4" s="81"/>
-      <c r="BW4" s="81"/>
-      <c r="BX4" s="81"/>
-      <c r="BY4" s="81"/>
-      <c r="BZ4" s="81">
+        <v>46167</v>
+      </c>
+      <c r="BT4" s="85"/>
+      <c r="BU4" s="85"/>
+      <c r="BV4" s="85"/>
+      <c r="BW4" s="85"/>
+      <c r="BX4" s="85"/>
+      <c r="BY4" s="85"/>
+      <c r="BZ4" s="85">
         <f>BZ5</f>
-        <v>46118</v>
-      </c>
-      <c r="CA4" s="81"/>
-      <c r="CB4" s="81"/>
-      <c r="CC4" s="81"/>
-      <c r="CD4" s="81"/>
-      <c r="CE4" s="81"/>
-      <c r="CF4" s="81"/>
-      <c r="CG4" s="81">
+        <v>46174</v>
+      </c>
+      <c r="CA4" s="85"/>
+      <c r="CB4" s="85"/>
+      <c r="CC4" s="85"/>
+      <c r="CD4" s="85"/>
+      <c r="CE4" s="85"/>
+      <c r="CF4" s="85"/>
+      <c r="CG4" s="85">
         <f>CG5</f>
-        <v>46125</v>
-      </c>
-      <c r="CH4" s="81"/>
-      <c r="CI4" s="81"/>
-      <c r="CJ4" s="81"/>
-      <c r="CK4" s="81"/>
-      <c r="CL4" s="81"/>
-      <c r="CM4" s="81"/>
-      <c r="CN4" s="81">
+        <v>46181</v>
+      </c>
+      <c r="CH4" s="85"/>
+      <c r="CI4" s="85"/>
+      <c r="CJ4" s="85"/>
+      <c r="CK4" s="85"/>
+      <c r="CL4" s="85"/>
+      <c r="CM4" s="85"/>
+      <c r="CN4" s="85">
         <f>CN5</f>
-        <v>46132</v>
-      </c>
-      <c r="CO4" s="81"/>
-      <c r="CP4" s="81"/>
-      <c r="CQ4" s="81"/>
-      <c r="CR4" s="81"/>
-      <c r="CS4" s="81"/>
-      <c r="CT4" s="81"/>
-      <c r="CU4" s="81">
+        <v>46188</v>
+      </c>
+      <c r="CO4" s="85"/>
+      <c r="CP4" s="85"/>
+      <c r="CQ4" s="85"/>
+      <c r="CR4" s="85"/>
+      <c r="CS4" s="85"/>
+      <c r="CT4" s="85"/>
+      <c r="CU4" s="85">
         <f>CU5</f>
-        <v>46139</v>
-      </c>
-      <c r="CV4" s="81"/>
-      <c r="CW4" s="81"/>
-      <c r="CX4" s="81"/>
-      <c r="CY4" s="81"/>
-      <c r="CZ4" s="81"/>
-      <c r="DA4" s="81"/>
-      <c r="DB4" s="81">
+        <v>46195</v>
+      </c>
+      <c r="CV4" s="85"/>
+      <c r="CW4" s="85"/>
+      <c r="CX4" s="85"/>
+      <c r="CY4" s="85"/>
+      <c r="CZ4" s="85"/>
+      <c r="DA4" s="85"/>
+      <c r="DB4" s="85">
         <f>DB5</f>
-        <v>46146</v>
-      </c>
-      <c r="DC4" s="81"/>
-      <c r="DD4" s="81"/>
-      <c r="DE4" s="81"/>
-      <c r="DF4" s="81"/>
-      <c r="DG4" s="81"/>
-      <c r="DH4" s="81"/>
-      <c r="DI4" s="81">
+        <v>46202</v>
+      </c>
+      <c r="DC4" s="85"/>
+      <c r="DD4" s="85"/>
+      <c r="DE4" s="85"/>
+      <c r="DF4" s="85"/>
+      <c r="DG4" s="85"/>
+      <c r="DH4" s="85"/>
+      <c r="DI4" s="85">
         <f>DI5</f>
-        <v>46153</v>
-      </c>
-      <c r="DJ4" s="81"/>
-      <c r="DK4" s="81"/>
-      <c r="DL4" s="81"/>
-      <c r="DM4" s="81"/>
-      <c r="DN4" s="81"/>
-      <c r="DO4" s="84"/>
+        <v>46209</v>
+      </c>
+      <c r="DJ4" s="85"/>
+      <c r="DK4" s="85"/>
+      <c r="DL4" s="85"/>
+      <c r="DM4" s="85"/>
+      <c r="DN4" s="85"/>
+      <c r="DO4" s="86"/>
     </row>
     <row r="5" spans="1:119" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="69"/>
@@ -1839,7 +1934,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="72" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D5" s="72" t="s">
         <v>2</v>
@@ -1849,451 +1944,451 @@
       </c>
       <c r="H5" s="21">
         <f>Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
-        <v>46048</v>
+        <v>46104</v>
       </c>
       <c r="I5" s="21">
         <f>H5+1</f>
-        <v>46049</v>
+        <v>46105</v>
       </c>
       <c r="J5" s="21">
         <f t="shared" ref="J5:AW5" si="0">I5+1</f>
-        <v>46050</v>
+        <v>46106</v>
       </c>
       <c r="K5" s="21">
         <f t="shared" si="0"/>
-        <v>46051</v>
+        <v>46107</v>
       </c>
       <c r="L5" s="21">
         <f t="shared" si="0"/>
-        <v>46052</v>
+        <v>46108</v>
       </c>
       <c r="M5" s="21">
         <f t="shared" si="0"/>
-        <v>46053</v>
+        <v>46109</v>
       </c>
       <c r="N5" s="22">
         <f t="shared" si="0"/>
-        <v>46054</v>
+        <v>46110</v>
       </c>
       <c r="O5" s="23">
         <f>N5+1</f>
-        <v>46055</v>
+        <v>46111</v>
       </c>
       <c r="P5" s="21">
         <f>O5+1</f>
-        <v>46056</v>
+        <v>46112</v>
       </c>
       <c r="Q5" s="21">
         <f t="shared" si="0"/>
-        <v>46057</v>
+        <v>46113</v>
       </c>
       <c r="R5" s="21">
         <f t="shared" si="0"/>
-        <v>46058</v>
+        <v>46114</v>
       </c>
       <c r="S5" s="21">
         <f t="shared" si="0"/>
-        <v>46059</v>
+        <v>46115</v>
       </c>
       <c r="T5" s="21">
         <f t="shared" si="0"/>
-        <v>46060</v>
+        <v>46116</v>
       </c>
       <c r="U5" s="22">
         <f t="shared" si="0"/>
-        <v>46061</v>
+        <v>46117</v>
       </c>
       <c r="V5" s="23">
         <f>U5+1</f>
-        <v>46062</v>
+        <v>46118</v>
       </c>
       <c r="W5" s="21">
         <f>V5+1</f>
-        <v>46063</v>
+        <v>46119</v>
       </c>
       <c r="X5" s="21">
         <f t="shared" si="0"/>
-        <v>46064</v>
+        <v>46120</v>
       </c>
       <c r="Y5" s="21">
         <f t="shared" si="0"/>
-        <v>46065</v>
+        <v>46121</v>
       </c>
       <c r="Z5" s="21">
         <f t="shared" si="0"/>
-        <v>46066</v>
+        <v>46122</v>
       </c>
       <c r="AA5" s="21">
         <f t="shared" si="0"/>
-        <v>46067</v>
+        <v>46123</v>
       </c>
       <c r="AB5" s="22">
         <f t="shared" si="0"/>
-        <v>46068</v>
+        <v>46124</v>
       </c>
       <c r="AC5" s="23">
         <f>AB5+1</f>
-        <v>46069</v>
+        <v>46125</v>
       </c>
       <c r="AD5" s="21">
         <f>AC5+1</f>
-        <v>46070</v>
+        <v>46126</v>
       </c>
       <c r="AE5" s="21">
         <f t="shared" si="0"/>
-        <v>46071</v>
+        <v>46127</v>
       </c>
       <c r="AF5" s="21">
         <f t="shared" si="0"/>
-        <v>46072</v>
+        <v>46128</v>
       </c>
       <c r="AG5" s="21">
         <f t="shared" si="0"/>
-        <v>46073</v>
+        <v>46129</v>
       </c>
       <c r="AH5" s="21">
         <f t="shared" si="0"/>
-        <v>46074</v>
+        <v>46130</v>
       </c>
       <c r="AI5" s="22">
         <f t="shared" si="0"/>
-        <v>46075</v>
+        <v>46131</v>
       </c>
       <c r="AJ5" s="23">
         <f>AI5+1</f>
-        <v>46076</v>
+        <v>46132</v>
       </c>
       <c r="AK5" s="21">
         <f>AJ5+1</f>
-        <v>46077</v>
+        <v>46133</v>
       </c>
       <c r="AL5" s="21">
         <f t="shared" si="0"/>
-        <v>46078</v>
+        <v>46134</v>
       </c>
       <c r="AM5" s="21">
         <f t="shared" si="0"/>
-        <v>46079</v>
+        <v>46135</v>
       </c>
       <c r="AN5" s="21">
         <f t="shared" si="0"/>
-        <v>46080</v>
+        <v>46136</v>
       </c>
       <c r="AO5" s="21">
         <f t="shared" si="0"/>
-        <v>46081</v>
+        <v>46137</v>
       </c>
       <c r="AP5" s="22">
         <f t="shared" si="0"/>
-        <v>46082</v>
+        <v>46138</v>
       </c>
       <c r="AQ5" s="23">
         <f>AP5+1</f>
-        <v>46083</v>
+        <v>46139</v>
       </c>
       <c r="AR5" s="21">
         <f>AQ5+1</f>
-        <v>46084</v>
+        <v>46140</v>
       </c>
       <c r="AS5" s="21">
         <f t="shared" si="0"/>
-        <v>46085</v>
+        <v>46141</v>
       </c>
       <c r="AT5" s="21">
         <f t="shared" si="0"/>
-        <v>46086</v>
+        <v>46142</v>
       </c>
       <c r="AU5" s="21">
         <f t="shared" si="0"/>
-        <v>46087</v>
+        <v>46143</v>
       </c>
       <c r="AV5" s="21">
         <f t="shared" si="0"/>
-        <v>46088</v>
+        <v>46144</v>
       </c>
       <c r="AW5" s="22">
         <f t="shared" si="0"/>
-        <v>46089</v>
+        <v>46145</v>
       </c>
       <c r="AX5" s="23">
         <f>AW5+1</f>
-        <v>46090</v>
+        <v>46146</v>
       </c>
       <c r="AY5" s="21">
         <f>AX5+1</f>
-        <v>46091</v>
+        <v>46147</v>
       </c>
       <c r="AZ5" s="21">
         <f t="shared" ref="AZ5:BD5" si="1">AY5+1</f>
-        <v>46092</v>
+        <v>46148</v>
       </c>
       <c r="BA5" s="21">
         <f t="shared" si="1"/>
-        <v>46093</v>
+        <v>46149</v>
       </c>
       <c r="BB5" s="21">
         <f t="shared" si="1"/>
-        <v>46094</v>
+        <v>46150</v>
       </c>
       <c r="BC5" s="21">
         <f t="shared" si="1"/>
-        <v>46095</v>
+        <v>46151</v>
       </c>
       <c r="BD5" s="22">
         <f t="shared" si="1"/>
-        <v>46096</v>
+        <v>46152</v>
       </c>
       <c r="BE5" s="23">
         <f>BD5+1</f>
-        <v>46097</v>
+        <v>46153</v>
       </c>
       <c r="BF5" s="21">
         <f>BE5+1</f>
-        <v>46098</v>
+        <v>46154</v>
       </c>
       <c r="BG5" s="21">
         <f t="shared" ref="BG5:BK5" si="2">BF5+1</f>
-        <v>46099</v>
+        <v>46155</v>
       </c>
       <c r="BH5" s="21">
         <f t="shared" si="2"/>
-        <v>46100</v>
+        <v>46156</v>
       </c>
       <c r="BI5" s="21">
         <f t="shared" si="2"/>
-        <v>46101</v>
+        <v>46157</v>
       </c>
       <c r="BJ5" s="21">
         <f t="shared" si="2"/>
-        <v>46102</v>
+        <v>46158</v>
       </c>
       <c r="BK5" s="53">
         <f t="shared" si="2"/>
-        <v>46103</v>
+        <v>46159</v>
       </c>
       <c r="BL5" s="21">
         <f>BK5+1</f>
-        <v>46104</v>
+        <v>46160</v>
       </c>
       <c r="BM5" s="21">
         <f>BL5+1</f>
-        <v>46105</v>
+        <v>46161</v>
       </c>
       <c r="BN5" s="21">
         <f t="shared" ref="BN5" si="3">BM5+1</f>
-        <v>46106</v>
+        <v>46162</v>
       </c>
       <c r="BO5" s="21">
         <f t="shared" ref="BO5" si="4">BN5+1</f>
-        <v>46107</v>
+        <v>46163</v>
       </c>
       <c r="BP5" s="21">
         <f t="shared" ref="BP5" si="5">BO5+1</f>
-        <v>46108</v>
+        <v>46164</v>
       </c>
       <c r="BQ5" s="21">
         <f t="shared" ref="BQ5" si="6">BP5+1</f>
-        <v>46109</v>
+        <v>46165</v>
       </c>
       <c r="BR5" s="22">
         <f t="shared" ref="BR5" si="7">BQ5+1</f>
-        <v>46110</v>
+        <v>46166</v>
       </c>
       <c r="BS5" s="23">
         <f>BR5+1</f>
-        <v>46111</v>
+        <v>46167</v>
       </c>
       <c r="BT5" s="21">
         <f>BS5+1</f>
-        <v>46112</v>
+        <v>46168</v>
       </c>
       <c r="BU5" s="21">
         <f t="shared" ref="BU5" si="8">BT5+1</f>
-        <v>46113</v>
+        <v>46169</v>
       </c>
       <c r="BV5" s="21">
         <f t="shared" ref="BV5" si="9">BU5+1</f>
-        <v>46114</v>
+        <v>46170</v>
       </c>
       <c r="BW5" s="21">
         <f t="shared" ref="BW5" si="10">BV5+1</f>
-        <v>46115</v>
+        <v>46171</v>
       </c>
       <c r="BX5" s="21">
         <f t="shared" ref="BX5" si="11">BW5+1</f>
-        <v>46116</v>
+        <v>46172</v>
       </c>
       <c r="BY5" s="22">
         <f t="shared" ref="BY5" si="12">BX5+1</f>
-        <v>46117</v>
+        <v>46173</v>
       </c>
       <c r="BZ5" s="23">
         <f>BY5+1</f>
-        <v>46118</v>
+        <v>46174</v>
       </c>
       <c r="CA5" s="21">
         <f>BZ5+1</f>
-        <v>46119</v>
+        <v>46175</v>
       </c>
       <c r="CB5" s="21">
         <f t="shared" ref="CB5" si="13">CA5+1</f>
-        <v>46120</v>
+        <v>46176</v>
       </c>
       <c r="CC5" s="21">
         <f t="shared" ref="CC5" si="14">CB5+1</f>
-        <v>46121</v>
+        <v>46177</v>
       </c>
       <c r="CD5" s="21">
         <f t="shared" ref="CD5" si="15">CC5+1</f>
-        <v>46122</v>
+        <v>46178</v>
       </c>
       <c r="CE5" s="21">
         <f t="shared" ref="CE5" si="16">CD5+1</f>
-        <v>46123</v>
+        <v>46179</v>
       </c>
       <c r="CF5" s="22">
         <f t="shared" ref="CF5" si="17">CE5+1</f>
-        <v>46124</v>
+        <v>46180</v>
       </c>
       <c r="CG5" s="23">
         <f>CF5+1</f>
-        <v>46125</v>
+        <v>46181</v>
       </c>
       <c r="CH5" s="21">
         <f>CG5+1</f>
-        <v>46126</v>
+        <v>46182</v>
       </c>
       <c r="CI5" s="21">
         <f t="shared" ref="CI5" si="18">CH5+1</f>
-        <v>46127</v>
+        <v>46183</v>
       </c>
       <c r="CJ5" s="21">
         <f t="shared" ref="CJ5" si="19">CI5+1</f>
-        <v>46128</v>
+        <v>46184</v>
       </c>
       <c r="CK5" s="21">
         <f t="shared" ref="CK5" si="20">CJ5+1</f>
-        <v>46129</v>
+        <v>46185</v>
       </c>
       <c r="CL5" s="21">
         <f t="shared" ref="CL5" si="21">CK5+1</f>
-        <v>46130</v>
+        <v>46186</v>
       </c>
       <c r="CM5" s="22">
         <f t="shared" ref="CM5" si="22">CL5+1</f>
-        <v>46131</v>
+        <v>46187</v>
       </c>
       <c r="CN5" s="23">
         <f>CM5+1</f>
-        <v>46132</v>
+        <v>46188</v>
       </c>
       <c r="CO5" s="21">
         <f>CN5+1</f>
-        <v>46133</v>
+        <v>46189</v>
       </c>
       <c r="CP5" s="21">
         <f t="shared" ref="CP5" si="23">CO5+1</f>
-        <v>46134</v>
+        <v>46190</v>
       </c>
       <c r="CQ5" s="21">
         <f t="shared" ref="CQ5" si="24">CP5+1</f>
-        <v>46135</v>
+        <v>46191</v>
       </c>
       <c r="CR5" s="21">
         <f t="shared" ref="CR5" si="25">CQ5+1</f>
-        <v>46136</v>
+        <v>46192</v>
       </c>
       <c r="CS5" s="21">
         <f t="shared" ref="CS5" si="26">CR5+1</f>
-        <v>46137</v>
+        <v>46193</v>
       </c>
       <c r="CT5" s="22">
         <f t="shared" ref="CT5" si="27">CS5+1</f>
-        <v>46138</v>
+        <v>46194</v>
       </c>
       <c r="CU5" s="23">
         <f>CT5+1</f>
-        <v>46139</v>
+        <v>46195</v>
       </c>
       <c r="CV5" s="21">
         <f>CU5+1</f>
-        <v>46140</v>
+        <v>46196</v>
       </c>
       <c r="CW5" s="21">
         <f t="shared" ref="CW5" si="28">CV5+1</f>
-        <v>46141</v>
+        <v>46197</v>
       </c>
       <c r="CX5" s="21">
         <f t="shared" ref="CX5" si="29">CW5+1</f>
-        <v>46142</v>
+        <v>46198</v>
       </c>
       <c r="CY5" s="21">
         <f t="shared" ref="CY5" si="30">CX5+1</f>
-        <v>46143</v>
+        <v>46199</v>
       </c>
       <c r="CZ5" s="21">
         <f t="shared" ref="CZ5" si="31">CY5+1</f>
-        <v>46144</v>
+        <v>46200</v>
       </c>
       <c r="DA5" s="22">
         <f t="shared" ref="DA5" si="32">CZ5+1</f>
-        <v>46145</v>
+        <v>46201</v>
       </c>
       <c r="DB5" s="23">
         <f>DA5+1</f>
-        <v>46146</v>
+        <v>46202</v>
       </c>
       <c r="DC5" s="21">
         <f>DB5+1</f>
-        <v>46147</v>
+        <v>46203</v>
       </c>
       <c r="DD5" s="21">
         <f t="shared" ref="DD5" si="33">DC5+1</f>
-        <v>46148</v>
+        <v>46204</v>
       </c>
       <c r="DE5" s="21">
         <f t="shared" ref="DE5" si="34">DD5+1</f>
-        <v>46149</v>
+        <v>46205</v>
       </c>
       <c r="DF5" s="21">
         <f t="shared" ref="DF5" si="35">DE5+1</f>
-        <v>46150</v>
+        <v>46206</v>
       </c>
       <c r="DG5" s="21">
         <f t="shared" ref="DG5" si="36">DF5+1</f>
-        <v>46151</v>
+        <v>46207</v>
       </c>
       <c r="DH5" s="22">
         <f t="shared" ref="DH5" si="37">DG5+1</f>
-        <v>46152</v>
+        <v>46208</v>
       </c>
       <c r="DI5" s="23">
         <f>DH5+1</f>
-        <v>46153</v>
+        <v>46209</v>
       </c>
       <c r="DJ5" s="21">
         <f>DI5+1</f>
-        <v>46154</v>
+        <v>46210</v>
       </c>
       <c r="DK5" s="21">
         <f t="shared" ref="DK5" si="38">DJ5+1</f>
-        <v>46155</v>
+        <v>46211</v>
       </c>
       <c r="DL5" s="21">
         <f t="shared" ref="DL5" si="39">DK5+1</f>
-        <v>46156</v>
+        <v>46212</v>
       </c>
       <c r="DM5" s="21">
         <f t="shared" ref="DM5" si="40">DL5+1</f>
-        <v>46157</v>
+        <v>46213</v>
       </c>
       <c r="DN5" s="21">
         <f t="shared" ref="DN5" si="41">DM5+1</f>
-        <v>46158</v>
+        <v>46214</v>
       </c>
       <c r="DO5" s="53">
         <f t="shared" ref="DO5" si="42">DN5+1</f>
-        <v>46159</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="6" spans="1:119" s="19" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2431,7 +2526,7 @@
         <v>T</v>
       </c>
       <c r="AN6" s="25" t="str">
-        <f t="shared" ref="AN6:CQ6" si="44">LEFT(TEXT(AN5,"ddd"),1)</f>
+        <f t="shared" ref="AN6:BK6" si="44">LEFT(TEXT(AN5,"ddd"),1)</f>
         <v>F</v>
       </c>
       <c r="AO6" s="25" t="str">
@@ -2527,227 +2622,227 @@
         <v>S</v>
       </c>
       <c r="BL6" s="24" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" ref="BL6:CQ6" si="45">LEFT(TEXT(BL5,"ddd"),1)</f>
         <v>M</v>
       </c>
       <c r="BM6" s="25" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>T</v>
       </c>
       <c r="BN6" s="25" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>W</v>
       </c>
       <c r="BO6" s="25" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>T</v>
       </c>
       <c r="BP6" s="25" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>F</v>
       </c>
       <c r="BQ6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="BR6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="BS6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>M</v>
-      </c>
-      <c r="BT6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="BU6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>W</v>
-      </c>
-      <c r="BV6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="BW6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>F</v>
-      </c>
-      <c r="BX6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="BY6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="BZ6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>M</v>
-      </c>
-      <c r="CA6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="CB6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>W</v>
-      </c>
-      <c r="CC6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="CD6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>F</v>
-      </c>
-      <c r="CE6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="CF6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="CG6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>M</v>
-      </c>
-      <c r="CH6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="CI6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>W</v>
-      </c>
-      <c r="CJ6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="CK6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>F</v>
-      </c>
-      <c r="CL6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="CM6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>S</v>
-      </c>
-      <c r="CN6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>M</v>
-      </c>
-      <c r="CO6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="CP6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>W</v>
-      </c>
-      <c r="CQ6" s="25" t="str">
-        <f t="shared" si="44"/>
-        <v>T</v>
-      </c>
-      <c r="CR6" s="25" t="str">
-        <f t="shared" ref="CR6:DO6" si="45">LEFT(TEXT(CR5,"ddd"),1)</f>
-        <v>F</v>
-      </c>
-      <c r="CS6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
-      <c r="CT6" s="25" t="str">
+      <c r="BR6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
-      <c r="CU6" s="25" t="str">
+      <c r="BS6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>M</v>
       </c>
-      <c r="CV6" s="25" t="str">
+      <c r="BT6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>T</v>
       </c>
-      <c r="CW6" s="25" t="str">
+      <c r="BU6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>W</v>
       </c>
-      <c r="CX6" s="25" t="str">
+      <c r="BV6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>T</v>
       </c>
-      <c r="CY6" s="25" t="str">
+      <c r="BW6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>F</v>
       </c>
-      <c r="CZ6" s="25" t="str">
+      <c r="BX6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
-      <c r="DA6" s="25" t="str">
+      <c r="BY6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
-      <c r="DB6" s="25" t="str">
+      <c r="BZ6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>M</v>
       </c>
-      <c r="DC6" s="25" t="str">
+      <c r="CA6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>T</v>
       </c>
-      <c r="DD6" s="25" t="str">
+      <c r="CB6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>W</v>
       </c>
-      <c r="DE6" s="25" t="str">
+      <c r="CC6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>T</v>
       </c>
-      <c r="DF6" s="25" t="str">
+      <c r="CD6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>F</v>
       </c>
-      <c r="DG6" s="25" t="str">
+      <c r="CE6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
-      <c r="DH6" s="25" t="str">
+      <c r="CF6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
-      <c r="DI6" s="25" t="str">
+      <c r="CG6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>M</v>
       </c>
-      <c r="DJ6" s="25" t="str">
+      <c r="CH6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>T</v>
       </c>
-      <c r="DK6" s="25" t="str">
+      <c r="CI6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>W</v>
       </c>
-      <c r="DL6" s="25" t="str">
+      <c r="CJ6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>T</v>
       </c>
-      <c r="DM6" s="25" t="str">
+      <c r="CK6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>F</v>
       </c>
-      <c r="DN6" s="25" t="str">
+      <c r="CL6" s="25" t="str">
         <f t="shared" si="45"/>
         <v>S</v>
       </c>
+      <c r="CM6" s="25" t="str">
+        <f t="shared" si="45"/>
+        <v>S</v>
+      </c>
+      <c r="CN6" s="25" t="str">
+        <f t="shared" si="45"/>
+        <v>M</v>
+      </c>
+      <c r="CO6" s="25" t="str">
+        <f t="shared" si="45"/>
+        <v>T</v>
+      </c>
+      <c r="CP6" s="25" t="str">
+        <f t="shared" si="45"/>
+        <v>W</v>
+      </c>
+      <c r="CQ6" s="25" t="str">
+        <f t="shared" si="45"/>
+        <v>T</v>
+      </c>
+      <c r="CR6" s="25" t="str">
+        <f t="shared" ref="CR6:DO6" si="46">LEFT(TEXT(CR5,"ddd"),1)</f>
+        <v>F</v>
+      </c>
+      <c r="CS6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
+      <c r="CT6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
+      <c r="CU6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>M</v>
+      </c>
+      <c r="CV6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>T</v>
+      </c>
+      <c r="CW6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>W</v>
+      </c>
+      <c r="CX6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>T</v>
+      </c>
+      <c r="CY6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>F</v>
+      </c>
+      <c r="CZ6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
+      <c r="DA6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
+      <c r="DB6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>M</v>
+      </c>
+      <c r="DC6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>T</v>
+      </c>
+      <c r="DD6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>W</v>
+      </c>
+      <c r="DE6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>T</v>
+      </c>
+      <c r="DF6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>F</v>
+      </c>
+      <c r="DG6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
+      <c r="DH6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
+      <c r="DI6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>M</v>
+      </c>
+      <c r="DJ6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>T</v>
+      </c>
+      <c r="DK6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>W</v>
+      </c>
+      <c r="DL6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>T</v>
+      </c>
+      <c r="DM6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>F</v>
+      </c>
+      <c r="DN6" s="25" t="str">
+        <f t="shared" si="46"/>
+        <v>S</v>
+      </c>
       <c r="DO6" s="54" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="46"/>
         <v>S</v>
       </c>
     </row>
@@ -2824,23 +2919,22 @@
     <row r="8" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="B8" s="30" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C8" s="61">
-        <f>E8-D8</f>
-        <v>5</v>
+        <f t="shared" ref="C8:C13" si="47">E8-D8</f>
+        <v>11</v>
       </c>
       <c r="D8" s="31">
-        <f>Project_Start</f>
-        <v>46050</v>
+        <v>46111</v>
       </c>
       <c r="E8" s="31">
-        <v>46055</v>
+        <v>46122</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="4">
-        <f t="shared" ref="G8:G14" si="46">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v>6</v>
+        <f t="shared" ref="G8:G16" si="48">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>12</v>
       </c>
       <c r="H8" s="32"/>
       <c r="I8" s="32"/>
@@ -2958,22 +3052,22 @@
     <row r="9" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
       <c r="B9" s="33" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C9" s="62">
-        <f>E9-D9</f>
-        <v>14</v>
+        <f t="shared" si="47"/>
+        <v>11</v>
       </c>
       <c r="D9" s="34">
-        <v>46062</v>
+        <v>46125</v>
       </c>
       <c r="E9" s="34">
-        <v>46076</v>
+        <v>46136</v>
       </c>
       <c r="F9" s="15"/>
       <c r="G9" s="4">
-        <f t="shared" si="46"/>
-        <v>15</v>
+        <f t="shared" si="48"/>
+        <v>12</v>
       </c>
       <c r="H9" s="32"/>
       <c r="I9" s="32"/>
@@ -3091,22 +3185,22 @@
     <row r="10" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="35" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C10" s="63">
-        <f>E10-D10</f>
-        <v>28</v>
+        <f t="shared" si="47"/>
+        <v>12</v>
       </c>
       <c r="D10" s="36">
-        <v>46078</v>
+        <v>46139</v>
       </c>
       <c r="E10" s="36">
-        <v>46106</v>
+        <v>46151</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="4">
-        <f t="shared" si="46"/>
-        <v>29</v>
+        <f t="shared" si="48"/>
+        <v>13</v>
       </c>
       <c r="H10" s="32"/>
       <c r="I10" s="32"/>
@@ -3224,22 +3318,22 @@
     <row r="11" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12"/>
       <c r="B11" s="37" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C11" s="64">
-        <f>E11-D11</f>
-        <v>25</v>
+        <f t="shared" si="47"/>
+        <v>33</v>
       </c>
       <c r="D11" s="38">
+        <v>46078</v>
+      </c>
+      <c r="E11" s="38">
         <v>46111</v>
-      </c>
-      <c r="E11" s="38">
-        <v>46136</v>
       </c>
       <c r="F11" s="15"/>
       <c r="G11" s="4">
-        <f t="shared" si="46"/>
-        <v>26</v>
+        <f t="shared" si="48"/>
+        <v>34</v>
       </c>
       <c r="H11" s="32"/>
       <c r="I11" s="32"/>
@@ -3357,22 +3451,22 @@
     <row r="12" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
       <c r="B12" s="58" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C12" s="65">
-        <f>E12-D12</f>
-        <v>19</v>
+        <f t="shared" si="47"/>
+        <v>25</v>
       </c>
       <c r="D12" s="59">
-        <v>46127</v>
+        <v>46111</v>
       </c>
       <c r="E12" s="59">
-        <v>46146</v>
+        <v>46136</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="4">
-        <f t="shared" si="46"/>
-        <v>20</v>
+        <f t="shared" si="48"/>
+        <v>26</v>
       </c>
       <c r="H12" s="32"/>
       <c r="I12" s="32"/>
@@ -3488,204 +3582,346 @@
       <c r="DO12" s="56"/>
     </row>
     <row r="13" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="61">
+        <f t="shared" si="47"/>
+        <v>19</v>
+      </c>
+      <c r="D13" s="31">
+        <v>46127</v>
+      </c>
+      <c r="E13" s="31">
+        <v>46146</v>
+      </c>
       <c r="F13" s="15"/>
-      <c r="G13" s="4" t="str">
-        <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-      <c r="K13" s="28"/>
-      <c r="L13" s="28"/>
-      <c r="M13" s="28"/>
-      <c r="N13" s="28"/>
-      <c r="O13" s="28"/>
-      <c r="P13" s="28"/>
-      <c r="Q13" s="28"/>
-      <c r="R13" s="28"/>
-      <c r="S13" s="28"/>
-      <c r="T13" s="28"/>
-      <c r="U13" s="28"/>
-      <c r="V13" s="28"/>
-      <c r="W13" s="28"/>
-      <c r="X13" s="28"/>
-      <c r="Y13" s="28"/>
-      <c r="Z13" s="28"/>
-      <c r="AA13" s="28"/>
-      <c r="AB13" s="28"/>
-      <c r="AC13" s="28"/>
-      <c r="AD13" s="28"/>
-      <c r="AE13" s="28"/>
-      <c r="AF13" s="28"/>
-      <c r="AG13" s="28"/>
-      <c r="AH13" s="28"/>
-      <c r="AI13" s="28"/>
-      <c r="AJ13" s="28"/>
-      <c r="AK13" s="28"/>
-      <c r="AL13" s="28"/>
-      <c r="AM13" s="28"/>
-      <c r="AN13" s="28"/>
-      <c r="AO13" s="28"/>
-      <c r="AP13" s="28"/>
-      <c r="AQ13" s="28"/>
-      <c r="AR13" s="28"/>
-      <c r="AS13" s="28"/>
-      <c r="AT13" s="28"/>
-      <c r="AU13" s="28"/>
-      <c r="AV13" s="28"/>
-      <c r="AW13" s="28"/>
-      <c r="AX13" s="28"/>
-      <c r="AY13" s="28"/>
-      <c r="AZ13" s="28"/>
-      <c r="BA13" s="28"/>
-      <c r="BB13" s="28"/>
-      <c r="BC13" s="28"/>
-      <c r="BD13" s="28"/>
-      <c r="BE13" s="28"/>
-      <c r="BF13" s="28"/>
-      <c r="BG13" s="28"/>
-      <c r="BH13" s="28"/>
-      <c r="BI13" s="28"/>
-      <c r="BJ13" s="28"/>
-      <c r="BK13" s="28"/>
+      <c r="G13" s="4">
+        <f t="shared" si="48"/>
+        <v>20</v>
+      </c>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
+      <c r="T13" s="32"/>
+      <c r="U13" s="32"/>
+      <c r="V13" s="32"/>
+      <c r="W13" s="32"/>
+      <c r="X13" s="32"/>
+      <c r="Y13" s="32"/>
+      <c r="Z13" s="32"/>
+      <c r="AA13" s="32"/>
+      <c r="AB13" s="32"/>
+      <c r="AC13" s="32"/>
+      <c r="AD13" s="32"/>
+      <c r="AE13" s="32"/>
+      <c r="AF13" s="32"/>
+      <c r="AG13" s="32"/>
+      <c r="AH13" s="32"/>
+      <c r="AI13" s="32"/>
+      <c r="AJ13" s="32"/>
+      <c r="AK13" s="32"/>
+      <c r="AL13" s="32"/>
+      <c r="AM13" s="32"/>
+      <c r="AN13" s="32"/>
+      <c r="AO13" s="32"/>
+      <c r="AP13" s="32"/>
+      <c r="AQ13" s="32"/>
+      <c r="AR13" s="32"/>
+      <c r="AS13" s="32"/>
+      <c r="AT13" s="32"/>
+      <c r="AU13" s="32"/>
+      <c r="AV13" s="32"/>
+      <c r="AW13" s="32"/>
+      <c r="AX13" s="32"/>
+      <c r="AY13" s="32"/>
+      <c r="AZ13" s="32"/>
+      <c r="BA13" s="32"/>
+      <c r="BB13" s="32"/>
+      <c r="BC13" s="32"/>
+      <c r="BD13" s="32"/>
+      <c r="BE13" s="32"/>
+      <c r="BF13" s="32"/>
+      <c r="BG13" s="32"/>
+      <c r="BH13" s="32"/>
+      <c r="BI13" s="32"/>
+      <c r="BJ13" s="32"/>
+      <c r="BK13" s="32"/>
+      <c r="BL13" s="32"/>
+      <c r="BM13" s="32"/>
+      <c r="BN13" s="32"/>
+      <c r="BO13" s="32"/>
+      <c r="BP13" s="32"/>
+      <c r="BQ13" s="32"/>
+      <c r="BR13" s="32"/>
+      <c r="BS13" s="32"/>
+      <c r="BT13" s="32"/>
+      <c r="BU13" s="32"/>
+      <c r="BV13" s="32"/>
+      <c r="BW13" s="32"/>
+      <c r="BX13" s="32"/>
+      <c r="BY13" s="32"/>
+      <c r="BZ13" s="32"/>
+      <c r="CA13" s="32"/>
+      <c r="CB13" s="32"/>
+      <c r="CC13" s="32"/>
+      <c r="CD13" s="32"/>
+      <c r="CE13" s="32"/>
+      <c r="CF13" s="32"/>
+      <c r="CG13" s="32"/>
+      <c r="CH13" s="32"/>
+      <c r="CI13" s="32"/>
+      <c r="CJ13" s="32"/>
+      <c r="CK13" s="32"/>
+      <c r="CL13" s="32"/>
+      <c r="CM13" s="32"/>
+      <c r="CN13" s="32"/>
+      <c r="CO13" s="32"/>
+      <c r="CP13" s="32"/>
+      <c r="CQ13" s="32"/>
+      <c r="CR13" s="32"/>
+      <c r="CS13" s="32"/>
+      <c r="CT13" s="32"/>
+      <c r="CU13" s="32"/>
+      <c r="CV13" s="32"/>
+      <c r="CW13" s="32"/>
+      <c r="CX13" s="32"/>
+      <c r="CY13" s="32"/>
+      <c r="CZ13" s="32"/>
+      <c r="DA13" s="32"/>
+      <c r="DB13" s="32"/>
+      <c r="DC13" s="32"/>
+      <c r="DD13" s="32"/>
+      <c r="DE13" s="32"/>
+      <c r="DF13" s="32"/>
+      <c r="DG13" s="32"/>
+      <c r="DH13" s="32"/>
+      <c r="DI13" s="32"/>
+      <c r="DJ13" s="32"/>
+      <c r="DK13" s="32"/>
+      <c r="DL13" s="32"/>
+      <c r="DM13" s="32"/>
+      <c r="DN13" s="32"/>
+      <c r="DO13" s="56"/>
     </row>
     <row r="14" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="41" t="s">
+      <c r="A14" s="12"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="4" t="str">
+        <f t="shared" si="48"/>
+        <v/>
+      </c>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="28"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="N14" s="28"/>
+      <c r="O14" s="28"/>
+      <c r="P14" s="28"/>
+      <c r="Q14" s="28"/>
+      <c r="R14" s="28"/>
+      <c r="S14" s="28"/>
+      <c r="T14" s="28"/>
+      <c r="U14" s="28"/>
+      <c r="V14" s="28"/>
+      <c r="W14" s="28"/>
+      <c r="X14" s="28"/>
+      <c r="Y14" s="28"/>
+      <c r="Z14" s="28"/>
+      <c r="AA14" s="28"/>
+      <c r="AB14" s="28"/>
+      <c r="AC14" s="28"/>
+      <c r="AD14" s="28"/>
+      <c r="AE14" s="28"/>
+      <c r="AF14" s="28"/>
+      <c r="AG14" s="28"/>
+      <c r="AH14" s="28"/>
+      <c r="AI14" s="28"/>
+      <c r="AJ14" s="28"/>
+      <c r="AK14" s="28"/>
+      <c r="AL14" s="28"/>
+      <c r="AM14" s="28"/>
+      <c r="AN14" s="28"/>
+      <c r="AO14" s="28"/>
+      <c r="AP14" s="28"/>
+      <c r="AQ14" s="28"/>
+      <c r="AR14" s="28"/>
+      <c r="AS14" s="28"/>
+      <c r="AT14" s="28"/>
+      <c r="AU14" s="28"/>
+      <c r="AV14" s="28"/>
+      <c r="AW14" s="28"/>
+      <c r="AX14" s="28"/>
+      <c r="AY14" s="28"/>
+      <c r="AZ14" s="28"/>
+      <c r="BA14" s="28"/>
+      <c r="BB14" s="28"/>
+      <c r="BC14" s="28"/>
+      <c r="BD14" s="28"/>
+      <c r="BE14" s="28"/>
+      <c r="BF14" s="28"/>
+      <c r="BG14" s="28"/>
+      <c r="BH14" s="28"/>
+      <c r="BI14" s="28"/>
+      <c r="BJ14" s="28"/>
+      <c r="BK14" s="28"/>
+    </row>
+    <row r="15" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:119" s="29" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13"/>
+      <c r="B16" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="5" t="str">
-        <f t="shared" si="46"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="5" t="str">
+        <f t="shared" si="48"/>
         <v/>
       </c>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44"/>
-      <c r="K14" s="44"/>
-      <c r="L14" s="44"/>
-      <c r="M14" s="44"/>
-      <c r="N14" s="44"/>
-      <c r="O14" s="44"/>
-      <c r="P14" s="44"/>
-      <c r="Q14" s="44"/>
-      <c r="R14" s="44"/>
-      <c r="S14" s="44"/>
-      <c r="T14" s="44"/>
-      <c r="U14" s="44"/>
-      <c r="V14" s="44"/>
-      <c r="W14" s="44"/>
-      <c r="X14" s="44"/>
-      <c r="Y14" s="44"/>
-      <c r="Z14" s="44"/>
-      <c r="AA14" s="44"/>
-      <c r="AB14" s="44"/>
-      <c r="AC14" s="44"/>
-      <c r="AD14" s="44"/>
-      <c r="AE14" s="44"/>
-      <c r="AF14" s="44"/>
-      <c r="AG14" s="44"/>
-      <c r="AH14" s="44"/>
-      <c r="AI14" s="44"/>
-      <c r="AJ14" s="44"/>
-      <c r="AK14" s="44"/>
-      <c r="AL14" s="44"/>
-      <c r="AM14" s="44"/>
-      <c r="AN14" s="44"/>
-      <c r="AO14" s="44"/>
-      <c r="AP14" s="44"/>
-      <c r="AQ14" s="44"/>
-      <c r="AR14" s="44"/>
-      <c r="AS14" s="44"/>
-      <c r="AT14" s="44"/>
-      <c r="AU14" s="44"/>
-      <c r="AV14" s="44"/>
-      <c r="AW14" s="44"/>
-      <c r="AX14" s="44"/>
-      <c r="AY14" s="44"/>
-      <c r="AZ14" s="44"/>
-      <c r="BA14" s="44"/>
-      <c r="BB14" s="44"/>
-      <c r="BC14" s="44"/>
-      <c r="BD14" s="44"/>
-      <c r="BE14" s="44"/>
-      <c r="BF14" s="44"/>
-      <c r="BG14" s="44"/>
-      <c r="BH14" s="44"/>
-      <c r="BI14" s="44"/>
-      <c r="BJ14" s="44"/>
-      <c r="BK14" s="44"/>
-      <c r="BL14" s="44"/>
-      <c r="BM14" s="44"/>
-      <c r="BN14" s="44"/>
-      <c r="BO14" s="44"/>
-      <c r="BP14" s="44"/>
-      <c r="BQ14" s="44"/>
-      <c r="BR14" s="44"/>
-      <c r="BS14" s="44"/>
-      <c r="BT14" s="44"/>
-      <c r="BU14" s="44"/>
-      <c r="BV14" s="44"/>
-      <c r="BW14" s="44"/>
-      <c r="BX14" s="44"/>
-      <c r="BY14" s="44"/>
-      <c r="BZ14" s="44"/>
-      <c r="CA14" s="44"/>
-      <c r="CB14" s="44"/>
-      <c r="CC14" s="44"/>
-      <c r="CD14" s="44"/>
-      <c r="CE14" s="44"/>
-      <c r="CF14" s="44"/>
-      <c r="CG14" s="44"/>
-      <c r="CH14" s="44"/>
-      <c r="CI14" s="44"/>
-      <c r="CJ14" s="44"/>
-      <c r="CK14" s="44"/>
-      <c r="CL14" s="44"/>
-      <c r="CM14" s="44"/>
-      <c r="CN14" s="44"/>
-      <c r="CO14" s="44"/>
-      <c r="CP14" s="44"/>
-      <c r="CQ14" s="44"/>
-      <c r="CR14" s="44"/>
-      <c r="CS14" s="44"/>
-      <c r="CT14" s="44"/>
-      <c r="CU14" s="44"/>
-      <c r="CV14" s="44"/>
-      <c r="CW14" s="44"/>
-      <c r="CX14" s="44"/>
-      <c r="CY14" s="44"/>
-      <c r="CZ14" s="44"/>
-      <c r="DA14" s="44"/>
-      <c r="DB14" s="44"/>
-      <c r="DC14" s="44"/>
-      <c r="DD14" s="44"/>
-      <c r="DE14" s="44"/>
-      <c r="DF14" s="44"/>
-      <c r="DG14" s="44"/>
-      <c r="DH14" s="44"/>
-      <c r="DI14" s="44"/>
-      <c r="DJ14" s="44"/>
-      <c r="DK14" s="44"/>
-      <c r="DL14" s="44"/>
-      <c r="DM14" s="44"/>
-      <c r="DN14" s="44"/>
-      <c r="DO14" s="44"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44"/>
+      <c r="K16" s="44"/>
+      <c r="L16" s="44"/>
+      <c r="M16" s="44"/>
+      <c r="N16" s="44"/>
+      <c r="O16" s="44"/>
+      <c r="P16" s="44"/>
+      <c r="Q16" s="44"/>
+      <c r="R16" s="44"/>
+      <c r="S16" s="44"/>
+      <c r="T16" s="44"/>
+      <c r="U16" s="44"/>
+      <c r="V16" s="44"/>
+      <c r="W16" s="44"/>
+      <c r="X16" s="44"/>
+      <c r="Y16" s="44"/>
+      <c r="Z16" s="44"/>
+      <c r="AA16" s="44"/>
+      <c r="AB16" s="44"/>
+      <c r="AC16" s="44"/>
+      <c r="AD16" s="44"/>
+      <c r="AE16" s="44"/>
+      <c r="AF16" s="44"/>
+      <c r="AG16" s="44"/>
+      <c r="AH16" s="44"/>
+      <c r="AI16" s="44"/>
+      <c r="AJ16" s="44"/>
+      <c r="AK16" s="44"/>
+      <c r="AL16" s="44"/>
+      <c r="AM16" s="44"/>
+      <c r="AN16" s="44"/>
+      <c r="AO16" s="44"/>
+      <c r="AP16" s="44"/>
+      <c r="AQ16" s="44"/>
+      <c r="AR16" s="44"/>
+      <c r="AS16" s="44"/>
+      <c r="AT16" s="44"/>
+      <c r="AU16" s="44"/>
+      <c r="AV16" s="44"/>
+      <c r="AW16" s="44"/>
+      <c r="AX16" s="44"/>
+      <c r="AY16" s="44"/>
+      <c r="AZ16" s="44"/>
+      <c r="BA16" s="44"/>
+      <c r="BB16" s="44"/>
+      <c r="BC16" s="44"/>
+      <c r="BD16" s="44"/>
+      <c r="BE16" s="44"/>
+      <c r="BF16" s="44"/>
+      <c r="BG16" s="44"/>
+      <c r="BH16" s="44"/>
+      <c r="BI16" s="44"/>
+      <c r="BJ16" s="44"/>
+      <c r="BK16" s="44"/>
+      <c r="BL16" s="44"/>
+      <c r="BM16" s="44"/>
+      <c r="BN16" s="44"/>
+      <c r="BO16" s="44"/>
+      <c r="BP16" s="44"/>
+      <c r="BQ16" s="44"/>
+      <c r="BR16" s="44"/>
+      <c r="BS16" s="44"/>
+      <c r="BT16" s="44"/>
+      <c r="BU16" s="44"/>
+      <c r="BV16" s="44"/>
+      <c r="BW16" s="44"/>
+      <c r="BX16" s="44"/>
+      <c r="BY16" s="44"/>
+      <c r="BZ16" s="44"/>
+      <c r="CA16" s="44"/>
+      <c r="CB16" s="44"/>
+      <c r="CC16" s="44"/>
+      <c r="CD16" s="44"/>
+      <c r="CE16" s="44"/>
+      <c r="CF16" s="44"/>
+      <c r="CG16" s="44"/>
+      <c r="CH16" s="44"/>
+      <c r="CI16" s="44"/>
+      <c r="CJ16" s="44"/>
+      <c r="CK16" s="44"/>
+      <c r="CL16" s="44"/>
+      <c r="CM16" s="44"/>
+      <c r="CN16" s="44"/>
+      <c r="CO16" s="44"/>
+      <c r="CP16" s="44"/>
+      <c r="CQ16" s="44"/>
+      <c r="CR16" s="44"/>
+      <c r="CS16" s="44"/>
+      <c r="CT16" s="44"/>
+      <c r="CU16" s="44"/>
+      <c r="CV16" s="44"/>
+      <c r="CW16" s="44"/>
+      <c r="CX16" s="44"/>
+      <c r="CY16" s="44"/>
+      <c r="CZ16" s="44"/>
+      <c r="DA16" s="44"/>
+      <c r="DB16" s="44"/>
+      <c r="DC16" s="44"/>
+      <c r="DD16" s="44"/>
+      <c r="DE16" s="44"/>
+      <c r="DF16" s="44"/>
+      <c r="DG16" s="44"/>
+      <c r="DH16" s="44"/>
+      <c r="DI16" s="44"/>
+      <c r="DJ16" s="44"/>
+      <c r="DK16" s="44"/>
+      <c r="DL16" s="44"/>
+      <c r="DM16" s="44"/>
+      <c r="DN16" s="44"/>
+      <c r="DO16" s="44"/>
     </row>
-    <row r="15" spans="1:119" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F15" s="3"/>
+    <row r="17" spans="5:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="3"/>
     </row>
-    <row r="16" spans="1:119" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E16" s="14"/>
+    <row r="18" spans="5:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -3716,44 +3952,64 @@
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="E5:E6"/>
   </mergeCells>
+  <conditionalFormatting sqref="H4:BK12 BL8:EO12 H10:EO13 BL4:DO6">
+    <cfRule type="expression" dxfId="16" priority="11">
+      <formula>AND(TODAY()&gt;=H$5, TODAY()&lt;I$5)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H8:EO8">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="15" priority="16">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="17" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:EO9">
-    <cfRule type="expression" dxfId="8" priority="6">
+  <conditionalFormatting sqref="H9:EO10">
+    <cfRule type="expression" dxfId="13" priority="14">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="15" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:EO10">
-    <cfRule type="expression" dxfId="6" priority="4">
+    <cfRule type="expression" dxfId="11" priority="5">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="6" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:EO11">
-    <cfRule type="expression" dxfId="4" priority="38">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="39" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="8" stopIfTrue="1">
+      <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="12">
+      <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="13" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:EO12 BL4:DO6 H4:BK11 BL8:EO11">
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>AND(TODAY()&gt;=H$5, TODAY()&lt;I$5)</formula>
+  <conditionalFormatting sqref="H12:EO12">
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="4" stopIfTrue="1">
+      <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="46">
+      <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="47" stopIfTrue="1">
+      <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:EO12">
+  <conditionalFormatting sqref="H13:EO13">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -3770,8 +4026,8 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter the name of the Project Lead in cell C3. Enter the Project Start date in cell Q1. Project Start: label is in cell I1." sqref="A3" xr:uid="{EEA7C783-457F-401F-98B9-9035587B9210}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="The Display week in cell Q2 is the starting week to display in the project schedule in cell I4. The project start date is Week 1. To change the display week, enter a new week number in cell Q2._x000a__x000a_Start date for each week is auto calculated starting in I4." sqref="A4" xr:uid="{43382715-6BC7-4B19-A31B-4B13A11ED166}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Cells I5 through BL5 contain the day number for the week represented in the cell block above each date and are auto calculated._x000a__x000a_Today's date is outlined from today's date in row 5 through the entire date column to the end of the project schedule." sqref="A5:A6" xr:uid="{7A3789A6-A3FB-43B6-A4F7-8C0AC564F67E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="B9 contains the task name.  C9 is the assignee.  D9 is a progress bar that shades based on the number entered into the cell.  _x000a__x000a_E9 contains the start date and F9 contains the end date._x000a__x000a_The Gantt chart will fill in starting in cell I9 based on task dates." sqref="A8 A12" xr:uid="{D870A2F6-6B07-4F5A-A81D-4BCCFADF8796}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row marks the end of the Project Schedule. DO NOT enter anything in this row. _x000a_Insert new rows ABOVE this one to continue building out your Project Schedule." sqref="A14" xr:uid="{79B9237E-4DD3-4E0F-8ED6-E0B695A99D96}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="B9 contains the task name.  C9 is the assignee.  D9 is a progress bar that shades based on the number entered into the cell.  _x000a__x000a_E9 contains the start date and F9 contains the end date._x000a__x000a_The Gantt chart will fill in starting in cell I9 based on task dates." sqref="A8 A12:A13" xr:uid="{D870A2F6-6B07-4F5A-A81D-4BCCFADF8796}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row marks the end of the Project Schedule. DO NOT enter anything in this row. _x000a_Insert new rows ABOVE this one to continue building out your Project Schedule." sqref="A16" xr:uid="{79B9237E-4DD3-4E0F-8ED6-E0B695A99D96}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
@@ -3827,7 +4083,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="55.2" x14ac:dyDescent="0.25">
       <c r="A9" s="48" t="s">
         <v>15</v>
       </c>

</xml_diff>